<commit_message>
chore: refresh dashboard template with buy ranges
</commit_message>
<xml_diff>
--- a/V2.8.5_ETF_A股统一决策仪表盘模板.xlsx
+++ b/V2.8.5_ETF_A股统一决策仪表盘模板.xlsx
@@ -27,7 +27,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'02_今日动作'!$A$1:$P$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_买入候选'!$A$1:$AM$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'03_买入候选'!$A$1:$AN$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'04_持仓风险'!$A$1:$AJ$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'05_年度配置'!$A$1:$S$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'06_组合总览'!$A$1:$B$38</definedName>
@@ -39,7 +39,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Positions'!$A$1:$AC$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Broker_Snapshot'!$A$1:$W$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Watchlist'!$A$1:$AB$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Framework_Rules'!$A$1:$D$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Framework_Rules'!$A$1:$D$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Checks'!$A$1:$G$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'使用说明'!$A$1:$C$10</definedName>
   </definedNames>
@@ -3007,19 +3007,11 @@
       <c r="J2" s="35" t="n"/>
       <c r="K2" s="35" t="n"/>
       <c r="L2" s="9" t="n"/>
-      <c r="M2" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N2" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M2" s="13" t="n"/>
+      <c r="N2" s="13" t="n"/>
       <c r="O2" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P2" s="13" t="n"/>
@@ -3080,19 +3072,11 @@
       <c r="J3" s="35" t="n"/>
       <c r="K3" s="35" t="n"/>
       <c r="L3" s="9" t="n"/>
-      <c r="M3" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N3" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M3" s="13" t="n"/>
+      <c r="N3" s="13" t="n"/>
       <c r="O3" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P3" s="13" t="n"/>
@@ -3153,19 +3137,11 @@
       <c r="J4" s="35" t="n"/>
       <c r="K4" s="35" t="n"/>
       <c r="L4" s="9" t="n"/>
-      <c r="M4" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N4" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M4" s="13" t="n"/>
+      <c r="N4" s="13" t="n"/>
       <c r="O4" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P4" s="13" t="n"/>
@@ -3226,19 +3202,11 @@
       <c r="J5" s="35" t="n"/>
       <c r="K5" s="35" t="n"/>
       <c r="L5" s="9" t="n"/>
-      <c r="M5" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N5" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M5" s="13" t="n"/>
+      <c r="N5" s="13" t="n"/>
       <c r="O5" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P5" s="13" t="n"/>
@@ -3299,19 +3267,11 @@
       <c r="J6" s="35" t="n"/>
       <c r="K6" s="35" t="n"/>
       <c r="L6" s="9" t="n"/>
-      <c r="M6" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N6" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M6" s="13" t="n"/>
+      <c r="N6" s="13" t="n"/>
       <c r="O6" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P6" s="13" t="n"/>
@@ -3372,19 +3332,11 @@
       <c r="J7" s="35" t="n"/>
       <c r="K7" s="35" t="n"/>
       <c r="L7" s="9" t="n"/>
-      <c r="M7" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N7" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M7" s="13" t="n"/>
+      <c r="N7" s="13" t="n"/>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>角色替代：核心持有（核心成长层）</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P7" s="13" t="n"/>
@@ -3453,19 +3405,11 @@
       <c r="J8" s="35" t="n"/>
       <c r="K8" s="35" t="n"/>
       <c r="L8" s="9" t="n"/>
-      <c r="M8" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N8" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M8" s="13" t="n"/>
+      <c r="N8" s="13" t="n"/>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>角色替代：核心持有（核心成长层）</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P8" s="13" t="n"/>
@@ -3534,19 +3478,11 @@
       <c r="J9" s="35" t="n"/>
       <c r="K9" s="35" t="n"/>
       <c r="L9" s="9" t="n"/>
-      <c r="M9" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N9" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M9" s="13" t="n"/>
+      <c r="N9" s="13" t="n"/>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P9" s="13" t="n"/>
@@ -3615,19 +3551,11 @@
       <c r="J10" s="35" t="n"/>
       <c r="K10" s="35" t="n"/>
       <c r="L10" s="9" t="n"/>
-      <c r="M10" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N10" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M10" s="13" t="n"/>
+      <c r="N10" s="13" t="n"/>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P10" s="13" t="n"/>
@@ -3688,19 +3616,11 @@
       <c r="J11" s="35" t="n"/>
       <c r="K11" s="35" t="n"/>
       <c r="L11" s="9" t="n"/>
-      <c r="M11" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N11" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M11" s="13" t="n"/>
+      <c r="N11" s="13" t="n"/>
       <c r="O11" s="13" t="inlineStr">
         <is>
-          <t>角色替代：战术仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P11" s="13" t="n"/>
@@ -3769,19 +3689,11 @@
       <c r="J12" s="35" t="n"/>
       <c r="K12" s="35" t="n"/>
       <c r="L12" s="9" t="n"/>
-      <c r="M12" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N12" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M12" s="13" t="n"/>
+      <c r="N12" s="13" t="n"/>
       <c r="O12" s="13" t="inlineStr">
         <is>
-          <t>角色替代：观察仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P12" s="13" t="n"/>
@@ -3850,19 +3762,11 @@
       <c r="J13" s="35" t="n"/>
       <c r="K13" s="35" t="n"/>
       <c r="L13" s="9" t="n"/>
-      <c r="M13" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N13" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M13" s="13" t="n"/>
+      <c r="N13" s="13" t="n"/>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>角色替代：低波权益层</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P13" s="13" t="n"/>
@@ -3931,19 +3835,11 @@
       <c r="J14" s="35" t="n"/>
       <c r="K14" s="35" t="n"/>
       <c r="L14" s="9" t="n"/>
-      <c r="M14" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N14" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M14" s="13" t="n"/>
+      <c r="N14" s="13" t="n"/>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>角色替代：防守资产（低波权益层）</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P14" s="13" t="n"/>
@@ -4012,19 +3908,11 @@
       <c r="J15" s="35" t="n"/>
       <c r="K15" s="35" t="n"/>
       <c r="L15" s="9" t="n"/>
-      <c r="M15" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N15" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M15" s="13" t="n"/>
+      <c r="N15" s="13" t="n"/>
       <c r="O15" s="13" t="inlineStr">
         <is>
-          <t>角色替代：防守资产（弹性低波层）</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P15" s="13" t="n"/>
@@ -4093,19 +3981,11 @@
       <c r="J16" s="35" t="n"/>
       <c r="K16" s="35" t="n"/>
       <c r="L16" s="9" t="n"/>
-      <c r="M16" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N16" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M16" s="13" t="n"/>
+      <c r="N16" s="13" t="n"/>
       <c r="O16" s="13" t="inlineStr">
         <is>
-          <t>角色替代：防守资产（纯防御层）</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P16" s="13" t="n"/>
@@ -4166,19 +4046,11 @@
       <c r="J17" s="35" t="n"/>
       <c r="K17" s="35" t="n"/>
       <c r="L17" s="9" t="n"/>
-      <c r="M17" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N17" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M17" s="13" t="n"/>
+      <c r="N17" s="13" t="n"/>
       <c r="O17" s="13" t="inlineStr">
         <is>
-          <t>角色替代：遗留仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P17" s="13" t="n"/>
@@ -4247,19 +4119,11 @@
       <c r="J18" s="35" t="n"/>
       <c r="K18" s="35" t="n"/>
       <c r="L18" s="9" t="n"/>
-      <c r="M18" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N18" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M18" s="13" t="n"/>
+      <c r="N18" s="13" t="n"/>
       <c r="O18" s="13" t="inlineStr">
         <is>
-          <t>角色替代：遗留仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P18" s="13" t="n"/>
@@ -4320,19 +4184,11 @@
       <c r="J19" s="35" t="n"/>
       <c r="K19" s="35" t="n"/>
       <c r="L19" s="9" t="n"/>
-      <c r="M19" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N19" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M19" s="13" t="n"/>
+      <c r="N19" s="13" t="n"/>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>角色替代：遗留仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P19" s="13" t="n"/>
@@ -4401,19 +4257,11 @@
       <c r="J20" s="35" t="n"/>
       <c r="K20" s="35" t="n"/>
       <c r="L20" s="9" t="n"/>
-      <c r="M20" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N20" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M20" s="13" t="n"/>
+      <c r="N20" s="13" t="n"/>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>角色替代：遗留仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P20" s="13" t="n"/>
@@ -4482,19 +4330,11 @@
       <c r="J21" s="35" t="n"/>
       <c r="K21" s="35" t="n"/>
       <c r="L21" s="9" t="n"/>
-      <c r="M21" s="13" t="inlineStr">
-        <is>
-          <t>量能替代：缺少成交额/20日均额</t>
-        </is>
-      </c>
-      <c r="N21" s="13" t="inlineStr">
-        <is>
-          <t>折溢价替代：缺少涨跌幅</t>
-        </is>
-      </c>
+      <c r="M21" s="13" t="n"/>
+      <c r="N21" s="13" t="n"/>
       <c r="O21" s="13" t="inlineStr">
         <is>
-          <t>角色替代：遗留仓</t>
+          <t>待填</t>
         </is>
       </c>
       <c r="P21" s="13" t="n"/>
@@ -9345,7 +9185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9489,66 +9329,66 @@
     <row r="7">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>情绪纪律</t>
+          <t>买点过滤</t>
         </is>
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>暂停新增</t>
+          <t>建议买入区间</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>情绪温度 ≥ 4</t>
+          <t>完整近期行情下按昨日低点与日内回踩区间复核；仓位已满仅保留观察区间；不自动下单</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>V2.8.5 第八部分</t>
+          <t>V2.8.4/V2.8.5 买点与行为纪律</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>执行纪律</t>
+          <t>情绪纪律</t>
         </is>
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>单日动作上限</t>
+          <t>暂停新增</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>一个买入方向 + 两个卖出/减仓方向</t>
+          <t>情绪温度 ≥ 4</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
         <is>
-          <t>V2.8.4/V2.8.5</t>
+          <t>V2.8.5 第八部分</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>现金安全垫</t>
+          <t>执行纪律</t>
         </is>
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>最低值</t>
+          <t>单日动作上限</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>300,000元</t>
+          <t>一个买入方向 + 两个卖出/减仓方向</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>V2.8.4 第十三部分</t>
+          <t>V2.8.4/V2.8.5</t>
         </is>
       </c>
     </row>
@@ -9560,12 +9400,12 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>目标值</t>
+          <t>最低值</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>500,000元</t>
+          <t>300,000元</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -9577,22 +9417,22 @@
     <row r="11">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>产业链簇上限</t>
+          <t>现金安全垫</t>
         </is>
       </c>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>半导体/芯片设备</t>
+          <t>目标值</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>≤ 18%</t>
+          <t>500,000元</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>V2.8.5 第四部分</t>
+          <t>V2.8.4 第十三部分</t>
         </is>
       </c>
     </row>
@@ -9604,12 +9444,12 @@
       </c>
       <c r="B12" s="13" t="inlineStr">
         <is>
-          <t>AI算力/云计算</t>
+          <t>半导体/芯片设备</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>≤ 15%</t>
+          <t>≤ 18%</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -9626,12 +9466,12 @@
       </c>
       <c r="B13" s="13" t="inlineStr">
         <is>
-          <t>机器人/自动化</t>
+          <t>AI算力/云计算</t>
         </is>
       </c>
       <c r="C13" s="9" t="inlineStr">
         <is>
-          <t>≤ 18%</t>
+          <t>≤ 15%</t>
         </is>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -9648,12 +9488,12 @@
       </c>
       <c r="B14" s="13" t="inlineStr">
         <is>
-          <t>新能源/绿电</t>
+          <t>机器人/自动化</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>≤ 25%</t>
+          <t>≤ 18%</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
@@ -9670,12 +9510,12 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>创新药/生物医药</t>
+          <t>新能源/绿电</t>
         </is>
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>≤ 15%</t>
+          <t>≤ 25%</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -9692,12 +9532,12 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>科技成长合计</t>
+          <t>创新药/生物医药</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>≤ 45%</t>
+          <t>≤ 15%</t>
         </is>
       </c>
       <c r="D16" s="9" t="inlineStr">
@@ -9709,22 +9549,22 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>第一年全资产配置</t>
+          <t>产业链簇上限</t>
         </is>
       </c>
       <c r="B17" s="13" t="inlineStr">
         <is>
-          <t>半导体设备ETF 159516</t>
+          <t>科技成长合计</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>目标8%；收益观察区间20%-30%</t>
+          <t>≤ 45%</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>1st年配置表.xlsx；缺口不是买入信号</t>
+          <t>V2.8.5 第四部分</t>
         </is>
       </c>
     </row>
@@ -9736,12 +9576,12 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>机器人ETF 562500</t>
+          <t>半导体设备ETF 159516</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>目标8%；收益观察区间18%-25%</t>
+          <t>目标8%；收益观察区间20%-30%</t>
         </is>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -9758,12 +9598,12 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>创业板人工智能ETF 159381</t>
+          <t>机器人ETF 562500</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>目标6%；收益观察区间20%-30%</t>
+          <t>目标8%；收益观察区间18%-25%</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
@@ -9780,12 +9620,12 @@
       </c>
       <c r="B20" s="13" t="inlineStr">
         <is>
-          <t>创新药ETF</t>
+          <t>创业板人工智能ETF 159381</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
         <is>
-          <t>目标2%；收益观察区间15%-25%</t>
+          <t>目标6%；收益观察区间20%-30%</t>
         </is>
       </c>
       <c r="D20" s="9" t="inlineStr">
@@ -9802,12 +9642,12 @@
       </c>
       <c r="B21" s="13" t="inlineStr">
         <is>
-          <t>比亚迪+绿电+储能</t>
+          <t>创新药ETF</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>目标3%；收益观察区间8%-15%</t>
+          <t>目标2%；收益观察区间15%-25%</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
@@ -9824,7 +9664,7 @@
       </c>
       <c r="B22" s="13" t="inlineStr">
         <is>
-          <t>云计算ETF</t>
+          <t>比亚迪+绿电+储能</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
@@ -9846,12 +9686,12 @@
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>中证A500ETF</t>
+          <t>云计算ETF</t>
         </is>
       </c>
       <c r="C23" s="9" t="inlineStr">
         <is>
-          <t>目标8%；收益观察区间6%-10%</t>
+          <t>目标3%；收益观察区间8%-15%</t>
         </is>
       </c>
       <c r="D23" s="9" t="inlineStr">
@@ -9868,12 +9708,12 @@
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>红利低波ETF</t>
+          <t>中证A500ETF</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>目标5%；收益观察区间5%-8%</t>
+          <t>目标8%；收益观察区间6%-10%</t>
         </is>
       </c>
       <c r="D24" s="9" t="inlineStr">
@@ -9890,12 +9730,12 @@
       </c>
       <c r="B25" s="13" t="inlineStr">
         <is>
-          <t>可转债ETF</t>
+          <t>红利低波ETF</t>
         </is>
       </c>
       <c r="C25" s="9" t="inlineStr">
         <is>
-          <t>目标10%；收益观察区间6%-10%</t>
+          <t>目标5%；收益观察区间5%-8%</t>
         </is>
       </c>
       <c r="D25" s="9" t="inlineStr">
@@ -9912,12 +9752,12 @@
       </c>
       <c r="B26" s="13" t="inlineStr">
         <is>
-          <t>战术机会仓</t>
+          <t>可转债ETF</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>目标3%；收益观察区间15%-30%</t>
+          <t>目标10%；收益观察区间6%-10%</t>
         </is>
       </c>
       <c r="D26" s="9" t="inlineStr">
@@ -9934,22 +9774,44 @@
       </c>
       <c r="B27" s="13" t="inlineStr">
         <is>
+          <t>战术机会仓</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>目标3%；收益观察区间15%-30%</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>1st年配置表.xlsx；缺口不是买入信号</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="13" t="inlineStr">
+        <is>
+          <t>第一年全资产配置</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
           <t>AI/半导体高质量个股篮子</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C28" s="9" t="inlineStr">
         <is>
           <t>目标2%；收益观察区间25%-35%</t>
         </is>
       </c>
-      <c r="D27" s="9" t="inlineStr">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>1st年配置表.xlsx；缺口不是买入信号</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D27"/>
+  <autoFilter ref="A1:D28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10756,48 +10618,49 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM20"/>
+  <dimension ref="A1:AN20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
-    <col width="11" customWidth="1" min="21" max="21"/>
-    <col width="10" customWidth="1" min="22" max="22"/>
-    <col width="13" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
-    <col width="16" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
-    <col width="16" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
-    <col width="16" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
-    <col width="36" customWidth="1" min="31" max="31"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="13" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="16" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="16" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
     <col width="36" customWidth="1" min="32" max="32"/>
     <col width="36" customWidth="1" min="33" max="33"/>
-    <col width="11" customWidth="1" min="34" max="34"/>
-    <col width="34" customWidth="1" min="35" max="35"/>
-    <col width="14" customWidth="1" min="36" max="36"/>
+    <col width="36" customWidth="1" min="34" max="34"/>
+    <col width="11" customWidth="1" min="35" max="35"/>
+    <col width="34" customWidth="1" min="36" max="36"/>
     <col width="14" customWidth="1" min="37" max="37"/>
     <col width="14" customWidth="1" min="38" max="38"/>
-    <col width="18" customWidth="1" min="39" max="39"/>
+    <col width="14" customWidth="1" min="39" max="39"/>
+    <col width="18" customWidth="1" min="40" max="40"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -10818,180 +10681,185 @@
       </c>
       <c r="D1" s="12" t="inlineStr">
         <is>
+          <t>建议买入区间</t>
+        </is>
+      </c>
+      <c r="E1" s="12" t="inlineStr">
+        <is>
           <t>建议</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="F1" s="12" t="inlineStr">
         <is>
           <t>阻断原因</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="G1" s="12" t="inlineStr">
         <is>
           <t>通过项</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>质量状态</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>市场权限</t>
         </is>
       </c>
-      <c r="I1" s="12" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>当前仓位</t>
         </is>
       </c>
-      <c r="J1" s="12" t="inlineStr">
+      <c r="K1" s="12" t="inlineStr">
         <is>
           <t>目标仓位</t>
         </is>
       </c>
-      <c r="K1" s="12" t="inlineStr">
+      <c r="L1" s="12" t="inlineStr">
         <is>
           <t>剩余额度</t>
         </is>
       </c>
-      <c r="L1" s="12" t="inlineStr">
+      <c r="M1" s="12" t="inlineStr">
         <is>
           <t>年度配置项</t>
         </is>
       </c>
-      <c r="M1" s="12" t="inlineStr">
+      <c r="N1" s="12" t="inlineStr">
         <is>
           <t>年度资金缺口</t>
         </is>
       </c>
-      <c r="N1" s="12" t="inlineStr">
+      <c r="O1" s="12" t="inlineStr">
         <is>
           <t>年度完成率</t>
         </is>
       </c>
-      <c r="O1" s="12" t="inlineStr">
+      <c r="P1" s="12" t="inlineStr">
         <is>
           <t>数据状态</t>
         </is>
       </c>
-      <c r="P1" s="12" t="inlineStr">
+      <c r="Q1" s="12" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
-      <c r="Q1" s="12" t="inlineStr">
+      <c r="R1" s="12" t="inlineStr">
         <is>
           <t>质量评分</t>
         </is>
       </c>
-      <c r="R1" s="12" t="inlineStr">
+      <c r="S1" s="12" t="inlineStr">
         <is>
           <t>情绪温度</t>
         </is>
       </c>
-      <c r="S1" s="12" t="inlineStr">
+      <c r="T1" s="12" t="inlineStr">
         <is>
           <t>反馈状态</t>
         </is>
       </c>
-      <c r="T1" s="12" t="inlineStr">
+      <c r="U1" s="12" t="inlineStr">
         <is>
           <t>仓位状态</t>
         </is>
       </c>
-      <c r="U1" s="12" t="inlineStr">
+      <c r="V1" s="12" t="inlineStr">
         <is>
           <t>Latest</t>
         </is>
       </c>
-      <c r="V1" s="12" t="inlineStr">
+      <c r="W1" s="12" t="inlineStr">
         <is>
           <t>PctChg</t>
         </is>
       </c>
-      <c r="W1" s="12" t="inlineStr">
+      <c r="X1" s="12" t="inlineStr">
         <is>
           <t>日内位置</t>
         </is>
       </c>
-      <c r="X1" s="12" t="inlineStr">
+      <c r="Y1" s="12" t="inlineStr">
         <is>
           <t>量能倍数</t>
         </is>
       </c>
-      <c r="Y1" s="12" t="inlineStr">
+      <c r="Z1" s="12" t="inlineStr">
         <is>
           <t>分时结构</t>
         </is>
       </c>
-      <c r="Z1" s="12" t="inlineStr">
+      <c r="AA1" s="12" t="inlineStr">
         <is>
           <t>量价关系</t>
         </is>
       </c>
-      <c r="AA1" s="12" t="inlineStr">
+      <c r="AB1" s="12" t="inlineStr">
         <is>
           <t>份额变动</t>
         </is>
       </c>
-      <c r="AB1" s="12" t="inlineStr">
+      <c r="AC1" s="12" t="inlineStr">
         <is>
           <t>折溢价</t>
         </is>
       </c>
-      <c r="AC1" s="12" t="inlineStr">
+      <c r="AD1" s="12" t="inlineStr">
         <is>
           <t>龙头同步</t>
         </is>
       </c>
-      <c r="AD1" s="12" t="inlineStr">
+      <c r="AE1" s="12" t="inlineStr">
         <is>
           <t>次日验证</t>
         </is>
       </c>
-      <c r="AE1" s="12" t="inlineStr">
+      <c r="AF1" s="12" t="inlineStr">
         <is>
           <t>通过明细</t>
         </is>
       </c>
-      <c r="AF1" s="12" t="inlineStr">
+      <c r="AG1" s="12" t="inlineStr">
         <is>
           <t>未通过项</t>
         </is>
       </c>
-      <c r="AG1" s="12" t="inlineStr">
+      <c r="AH1" s="12" t="inlineStr">
         <is>
           <t>待确认项</t>
         </is>
       </c>
-      <c r="AH1" s="12" t="inlineStr">
+      <c r="AI1" s="12" t="inlineStr">
         <is>
           <t>一票否决</t>
         </is>
       </c>
-      <c r="AI1" s="12" t="inlineStr">
+      <c r="AJ1" s="12" t="inlineStr">
         <is>
           <t>否决原因</t>
         </is>
       </c>
-      <c r="AJ1" s="12" t="inlineStr">
+      <c r="AK1" s="12" t="inlineStr">
         <is>
           <t>年度全资产目标</t>
         </is>
       </c>
-      <c r="AK1" s="12" t="inlineStr">
+      <c r="AL1" s="12" t="inlineStr">
         <is>
           <t>年度目标金额</t>
         </is>
       </c>
-      <c r="AL1" s="12" t="inlineStr">
+      <c r="AM1" s="12" t="inlineStr">
         <is>
           <t>年度组内当前金额</t>
         </is>
       </c>
-      <c r="AM1" s="12" t="inlineStr">
+      <c r="AN1" s="12" t="inlineStr">
         <is>
           <t>年度配置状态</t>
         </is>
@@ -11015,142 +10883,147 @@
       </c>
       <c r="D2" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E2" s="20" t="inlineStr">
+        <is>
           <t>质量评分或证据不完整，先补评分，禁止新增</t>
         </is>
       </c>
-      <c r="E2" s="21" t="inlineStr">
+      <c r="F2" s="21" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="F2" s="21" t="n">
+      <c r="G2" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="20" t="inlineStr">
+      <c r="H2" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H2" s="21" t="inlineStr">
+      <c r="I2" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I2" s="22" t="n">
+      <c r="J2" s="22" t="n">
         <v>0</v>
-      </c>
-      <c r="J2" s="22" t="n">
-        <v>0.03</v>
       </c>
       <c r="K2" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="L2" s="20" t="inlineStr">
+      <c r="L2" s="22" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="M2" s="20" t="inlineStr">
         <is>
           <t>创新药ETF</t>
         </is>
       </c>
-      <c r="M2" s="23" t="n">
+      <c r="N2" s="23" t="n">
         <v>95660</v>
       </c>
-      <c r="N2" s="22" t="n">
+      <c r="O2" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="O2" s="21" t="inlineStr">
+      <c r="P2" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P2" s="21" t="inlineStr">
+      <c r="Q2" s="21" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q2" s="24" t="n"/>
-      <c r="R2" s="21" t="n">
+      <c r="R2" s="24" t="n"/>
+      <c r="S2" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S2" s="21" t="inlineStr">
+      <c r="T2" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T2" s="20" t="inlineStr">
+      <c r="U2" s="20" t="inlineStr">
         <is>
           <t>低于目标，剩余 3.00%</t>
         </is>
       </c>
-      <c r="U2" s="25" t="n">
-        <v/>
-      </c>
-      <c r="V2" s="26" t="n"/>
-      <c r="W2" s="21" t="n"/>
-      <c r="X2" s="26" t="n"/>
-      <c r="Y2" s="21" t="inlineStr">
+      <c r="V2" s="25" t="n">
+        <v/>
+      </c>
+      <c r="W2" s="26" t="n"/>
+      <c r="X2" s="21" t="n"/>
+      <c r="Y2" s="26" t="n"/>
+      <c r="Z2" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z2" s="20" t="inlineStr">
+      <c r="AA2" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA2" s="21" t="inlineStr">
+      <c r="AB2" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB2" s="21" t="inlineStr">
+      <c r="AC2" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC2" s="21" t="inlineStr">
+      <c r="AD2" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD2" s="20" t="inlineStr">
+      <c r="AE2" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE2" s="20" t="inlineStr">
+      <c r="AF2" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF2" s="20" t="inlineStr">
+      <c r="AG2" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG2" s="20" t="inlineStr">
+      <c r="AH2" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH2" s="14" t="inlineStr">
+      <c r="AI2" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI2" s="20" t="inlineStr">
+      <c r="AJ2" s="20" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="AJ2" s="22" t="n">
+      <c r="AK2" s="22" t="n">
         <v>0.02</v>
       </c>
-      <c r="AK2" s="23" t="n">
+      <c r="AL2" s="23" t="n">
         <v>95660</v>
       </c>
-      <c r="AL2" s="23" t="n">
+      <c r="AM2" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="AM2" s="20" t="inlineStr">
+      <c r="AN2" s="20" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -11174,142 +11047,147 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
           <t>质量评分或证据不完整，先补评分，禁止新增</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="F3" s="13" t="n">
+      <c r="G3" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="H3" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="I3" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I3" s="16" t="n">
+      <c r="J3" s="16" t="n">
         <v>0.0406</v>
       </c>
-      <c r="J3" s="16" t="n">
+      <c r="K3" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="K3" s="16" t="n">
+      <c r="L3" s="16" t="n">
         <v>0.009400000000000006</v>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t>红利低波ETF</t>
         </is>
       </c>
-      <c r="M3" s="17" t="n">
+      <c r="N3" s="17" t="n">
         <v>196780</v>
       </c>
-      <c r="N3" s="16" t="n">
+      <c r="O3" s="16" t="n">
         <v>0.1771691407066694</v>
       </c>
-      <c r="O3" s="13" t="inlineStr">
+      <c r="P3" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P3" s="13" t="inlineStr">
+      <c r="Q3" s="13" t="inlineStr">
         <is>
           <t>低波权益层</t>
         </is>
       </c>
-      <c r="Q3" s="27" t="n"/>
-      <c r="R3" s="13" t="n">
+      <c r="R3" s="27" t="n"/>
+      <c r="S3" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S3" s="13" t="inlineStr">
+      <c r="T3" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T3" s="9" t="inlineStr">
+      <c r="U3" s="9" t="inlineStr">
         <is>
           <t>低于目标，剩余 0.94%</t>
         </is>
       </c>
-      <c r="U3" s="28" t="n">
+      <c r="V3" s="28" t="n">
         <v>1.115</v>
       </c>
-      <c r="V3" s="29" t="n"/>
-      <c r="W3" s="13" t="n"/>
-      <c r="X3" s="29" t="n"/>
-      <c r="Y3" s="13" t="inlineStr">
+      <c r="W3" s="29" t="n"/>
+      <c r="X3" s="13" t="n"/>
+      <c r="Y3" s="29" t="n"/>
+      <c r="Z3" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z3" s="9" t="inlineStr">
+      <c r="AA3" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA3" s="13" t="inlineStr">
+      <c r="AB3" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB3" s="13" t="inlineStr">
+      <c r="AC3" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC3" s="13" t="inlineStr">
+      <c r="AD3" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD3" s="9" t="inlineStr">
+      <c r="AE3" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE3" s="9" t="inlineStr">
+      <c r="AF3" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF3" s="9" t="inlineStr">
+      <c r="AG3" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG3" s="9" t="inlineStr">
+      <c r="AH3" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH3" s="14" t="inlineStr">
+      <c r="AI3" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI3" s="9" t="inlineStr">
+      <c r="AJ3" s="9" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="AJ3" s="16" t="n">
+      <c r="AK3" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="AK3" s="17" t="n">
+      <c r="AL3" s="17" t="n">
         <v>239150</v>
       </c>
-      <c r="AL3" s="17" t="n">
+      <c r="AM3" s="17" t="n">
         <v>42370</v>
       </c>
-      <c r="AM3" s="9" t="inlineStr">
+      <c r="AN3" s="9" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -11333,142 +11211,147 @@
       </c>
       <c r="D4" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E4" s="20" t="inlineStr">
+        <is>
           <t>持有不加，禁止新增；低于目标，剩余 0.65%</t>
         </is>
       </c>
-      <c r="E4" s="21" t="inlineStr">
+      <c r="F4" s="21" t="inlineStr">
         <is>
           <t>持有不加，禁止新增仓位</t>
         </is>
       </c>
-      <c r="F4" s="21" t="n">
+      <c r="G4" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="H4" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H4" s="21" t="inlineStr">
+      <c r="I4" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="J4" s="22" t="n">
         <v>0.1335</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="K4" s="22" t="n">
         <v>0.14</v>
       </c>
-      <c r="K4" s="22" t="n">
+      <c r="L4" s="22" t="n">
         <v>0.006500000000000006</v>
       </c>
-      <c r="L4" s="20" t="inlineStr">
+      <c r="M4" s="20" t="inlineStr">
         <is>
           <t>机器人ETF 562500</t>
         </is>
       </c>
-      <c r="M4" s="23" t="n">
+      <c r="N4" s="23" t="n">
         <v>243180.8</v>
       </c>
-      <c r="N4" s="22" t="n">
+      <c r="O4" s="22" t="n">
         <v>0.364465816433201</v>
       </c>
-      <c r="O4" s="21" t="inlineStr">
+      <c r="P4" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P4" s="21" t="inlineStr">
+      <c r="Q4" s="21" t="inlineStr">
         <is>
           <t>核心成长层</t>
         </is>
       </c>
-      <c r="Q4" s="24" t="n"/>
-      <c r="R4" s="21" t="n">
+      <c r="R4" s="24" t="n"/>
+      <c r="S4" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S4" s="21" t="inlineStr">
+      <c r="T4" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T4" s="20" t="inlineStr">
+      <c r="U4" s="20" t="inlineStr">
         <is>
           <t>低于目标，剩余 0.65%</t>
         </is>
       </c>
-      <c r="U4" s="25" t="n">
+      <c r="V4" s="25" t="n">
         <v>1.168</v>
       </c>
-      <c r="V4" s="26" t="n"/>
-      <c r="W4" s="21" t="n"/>
-      <c r="X4" s="26" t="n"/>
-      <c r="Y4" s="21" t="inlineStr">
+      <c r="W4" s="26" t="n"/>
+      <c r="X4" s="21" t="n"/>
+      <c r="Y4" s="26" t="n"/>
+      <c r="Z4" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z4" s="20" t="inlineStr">
+      <c r="AA4" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA4" s="21" t="inlineStr">
+      <c r="AB4" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB4" s="21" t="inlineStr">
+      <c r="AC4" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC4" s="21" t="inlineStr">
+      <c r="AD4" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD4" s="20" t="inlineStr">
+      <c r="AE4" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE4" s="20" t="inlineStr">
+      <c r="AF4" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF4" s="20" t="inlineStr">
+      <c r="AG4" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG4" s="20" t="inlineStr">
+      <c r="AH4" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH4" s="14" t="inlineStr">
+      <c r="AI4" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI4" s="20" t="inlineStr">
+      <c r="AJ4" s="20" t="inlineStr">
         <is>
           <t>持有不加，禁止新增仓位</t>
         </is>
       </c>
-      <c r="AJ4" s="22" t="n">
+      <c r="AK4" s="22" t="n">
         <v>0.08</v>
       </c>
-      <c r="AK4" s="23" t="n">
+      <c r="AL4" s="23" t="n">
         <v>382640</v>
       </c>
-      <c r="AL4" s="23" t="n">
+      <c r="AM4" s="23" t="n">
         <v>139459.2</v>
       </c>
-      <c r="AM4" s="20" t="inlineStr">
+      <c r="AN4" s="20" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -11492,138 +11375,143 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
           <t>质量评分或证据不完整，先补评分，禁止新增</t>
         </is>
       </c>
-      <c r="E5" s="13" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="G5" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="I5" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I5" s="16" t="n">
+      <c r="J5" s="16" t="n">
         <v>0</v>
-      </c>
-      <c r="J5" s="16" t="n">
-        <v>0.005</v>
       </c>
       <c r="K5" s="16" t="n">
         <v>0.005</v>
       </c>
-      <c r="L5" s="9" t="n"/>
-      <c r="M5" s="17" t="n">
-        <v/>
-      </c>
-      <c r="N5" s="16" t="n">
-        <v/>
-      </c>
-      <c r="O5" s="13" t="inlineStr">
+      <c r="L5" s="16" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="17" t="n">
+        <v/>
+      </c>
+      <c r="O5" s="16" t="n">
+        <v/>
+      </c>
+      <c r="P5" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P5" s="13" t="inlineStr">
+      <c r="Q5" s="13" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q5" s="27" t="n"/>
-      <c r="R5" s="13" t="n">
+      <c r="R5" s="27" t="n"/>
+      <c r="S5" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S5" s="13" t="inlineStr">
+      <c r="T5" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T5" s="9" t="inlineStr">
+      <c r="U5" s="9" t="inlineStr">
         <is>
           <t>低于目标，剩余 0.50%</t>
         </is>
       </c>
-      <c r="U5" s="28" t="n">
-        <v/>
-      </c>
-      <c r="V5" s="29" t="n"/>
-      <c r="W5" s="13" t="n"/>
-      <c r="X5" s="29" t="n"/>
-      <c r="Y5" s="13" t="inlineStr">
+      <c r="V5" s="28" t="n">
+        <v/>
+      </c>
+      <c r="W5" s="29" t="n"/>
+      <c r="X5" s="13" t="n"/>
+      <c r="Y5" s="29" t="n"/>
+      <c r="Z5" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z5" s="9" t="inlineStr">
+      <c r="AA5" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA5" s="13" t="inlineStr">
+      <c r="AB5" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB5" s="13" t="inlineStr">
+      <c r="AC5" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC5" s="13" t="inlineStr">
+      <c r="AD5" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD5" s="9" t="inlineStr">
+      <c r="AE5" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE5" s="9" t="inlineStr">
+      <c r="AF5" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF5" s="9" t="inlineStr">
+      <c r="AG5" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG5" s="9" t="inlineStr">
+      <c r="AH5" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH5" s="14" t="inlineStr">
+      <c r="AI5" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI5" s="9" t="inlineStr">
+      <c r="AJ5" s="9" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="AJ5" s="16" t="n">
-        <v/>
-      </c>
-      <c r="AK5" s="17" t="n">
+      <c r="AK5" s="16" t="n">
         <v/>
       </c>
       <c r="AL5" s="17" t="n">
         <v/>
       </c>
-      <c r="AM5" s="9" t="n"/>
+      <c r="AM5" s="17" t="n">
+        <v/>
+      </c>
+      <c r="AN5" s="9" t="n"/>
     </row>
     <row r="6" ht="38" customHeight="1">
       <c r="A6" s="18" t="inlineStr">
@@ -11643,142 +11531,147 @@
       </c>
       <c r="D6" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
           <t>质量评分或证据不完整，先补评分，禁止新增</t>
         </is>
       </c>
-      <c r="E6" s="21" t="inlineStr">
+      <c r="F6" s="21" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="G6" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="H6" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H6" s="21" t="inlineStr">
+      <c r="I6" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I6" s="22" t="n">
+      <c r="J6" s="22" t="n">
         <v>0.0369</v>
       </c>
-      <c r="J6" s="22" t="n">
+      <c r="K6" s="22" t="n">
         <v>0.04</v>
       </c>
-      <c r="K6" s="22" t="n">
+      <c r="L6" s="22" t="n">
         <v>0.003099999999999999</v>
       </c>
-      <c r="L6" s="20" t="inlineStr">
+      <c r="M6" s="20" t="inlineStr">
         <is>
           <t>可转债ETF</t>
         </is>
       </c>
-      <c r="M6" s="23" t="n">
+      <c r="N6" s="23" t="n">
         <v>439801</v>
       </c>
-      <c r="N6" s="22" t="n">
+      <c r="O6" s="22" t="n">
         <v>0.08049132343717333</v>
       </c>
-      <c r="O6" s="21" t="inlineStr">
+      <c r="P6" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P6" s="21" t="inlineStr">
+      <c r="Q6" s="21" t="inlineStr">
         <is>
           <t>弹性低波层</t>
         </is>
       </c>
-      <c r="Q6" s="24" t="n"/>
-      <c r="R6" s="21" t="n">
+      <c r="R6" s="24" t="n"/>
+      <c r="S6" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S6" s="21" t="inlineStr">
+      <c r="T6" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T6" s="20" t="inlineStr">
+      <c r="U6" s="20" t="inlineStr">
         <is>
           <t>低于目标，剩余 0.31%</t>
         </is>
       </c>
-      <c r="U6" s="25" t="n">
+      <c r="V6" s="25" t="n">
         <v>12.833</v>
       </c>
-      <c r="V6" s="26" t="n"/>
-      <c r="W6" s="21" t="n"/>
-      <c r="X6" s="26" t="n"/>
-      <c r="Y6" s="21" t="inlineStr">
+      <c r="W6" s="26" t="n"/>
+      <c r="X6" s="21" t="n"/>
+      <c r="Y6" s="26" t="n"/>
+      <c r="Z6" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z6" s="20" t="inlineStr">
+      <c r="AA6" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA6" s="21" t="inlineStr">
+      <c r="AB6" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB6" s="21" t="inlineStr">
+      <c r="AC6" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC6" s="21" t="inlineStr">
+      <c r="AD6" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD6" s="20" t="inlineStr">
+      <c r="AE6" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE6" s="20" t="inlineStr">
+      <c r="AF6" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF6" s="20" t="inlineStr">
+      <c r="AG6" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG6" s="20" t="inlineStr">
+      <c r="AH6" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH6" s="14" t="inlineStr">
+      <c r="AI6" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI6" s="20" t="inlineStr">
+      <c r="AJ6" s="20" t="inlineStr">
         <is>
           <t>缺少完整质量评分或证据，禁止新增</t>
         </is>
       </c>
-      <c r="AJ6" s="22" t="n">
+      <c r="AK6" s="22" t="n">
         <v>0.1</v>
       </c>
-      <c r="AK6" s="23" t="n">
+      <c r="AL6" s="23" t="n">
         <v>478300</v>
       </c>
-      <c r="AL6" s="23" t="n">
+      <c r="AM6" s="23" t="n">
         <v>38499</v>
       </c>
-      <c r="AM6" s="20" t="inlineStr">
+      <c r="AN6" s="20" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -11802,142 +11695,147 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
           <t>超目标 0.80%，禁止加仓</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="F7" s="13" t="n">
+      <c r="G7" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="H7" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H7" s="13" t="inlineStr">
+      <c r="I7" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I7" s="16" t="n">
+      <c r="J7" s="16" t="n">
         <v>0.058</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="K7" s="16" t="n">
         <v>0.05</v>
       </c>
-      <c r="K7" s="16" t="n">
+      <c r="L7" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>半导体设备ETF 159516</t>
         </is>
       </c>
-      <c r="M7" s="17" t="n">
+      <c r="N7" s="17" t="n">
         <v>322000</v>
       </c>
-      <c r="N7" s="16" t="n">
+      <c r="O7" s="16" t="n">
         <v>0.158477942713778</v>
       </c>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="P7" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P7" s="13" t="inlineStr">
+      <c r="Q7" s="13" t="inlineStr">
         <is>
           <t>核心成长层</t>
         </is>
       </c>
-      <c r="Q7" s="27" t="n"/>
-      <c r="R7" s="13" t="n">
+      <c r="R7" s="27" t="n"/>
+      <c r="S7" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S7" s="13" t="inlineStr">
+      <c r="T7" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T7" s="9" t="inlineStr">
+      <c r="U7" s="9" t="inlineStr">
         <is>
           <t>超目标 0.80%</t>
         </is>
       </c>
-      <c r="U7" s="28" t="n">
+      <c r="V7" s="28" t="n">
         <v>1.516</v>
       </c>
-      <c r="V7" s="29" t="n"/>
-      <c r="W7" s="13" t="n"/>
-      <c r="X7" s="29" t="n"/>
-      <c r="Y7" s="13" t="inlineStr">
+      <c r="W7" s="29" t="n"/>
+      <c r="X7" s="13" t="n"/>
+      <c r="Y7" s="29" t="n"/>
+      <c r="Z7" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z7" s="9" t="inlineStr">
+      <c r="AA7" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA7" s="13" t="inlineStr">
+      <c r="AB7" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB7" s="13" t="inlineStr">
+      <c r="AC7" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC7" s="13" t="inlineStr">
+      <c r="AD7" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD7" s="9" t="inlineStr">
+      <c r="AE7" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE7" s="9" t="inlineStr">
+      <c r="AF7" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF7" s="9" t="inlineStr">
+      <c r="AG7" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG7" s="9" t="inlineStr">
+      <c r="AH7" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH7" s="14" t="inlineStr">
+      <c r="AI7" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI7" s="9" t="inlineStr">
+      <c r="AJ7" s="9" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="AJ7" s="16" t="n">
+      <c r="AK7" s="16" t="n">
         <v>0.08</v>
       </c>
-      <c r="AK7" s="17" t="n">
+      <c r="AL7" s="17" t="n">
         <v>382640</v>
       </c>
-      <c r="AL7" s="17" t="n">
+      <c r="AM7" s="17" t="n">
         <v>60640</v>
       </c>
-      <c r="AM7" s="9" t="inlineStr">
+      <c r="AN7" s="9" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -11961,142 +11859,147 @@
       </c>
       <c r="D8" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
           <t>超目标 0.07%，禁止加仓</t>
         </is>
       </c>
-      <c r="E8" s="21" t="inlineStr">
+      <c r="F8" s="21" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="G8" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H8" s="21" t="inlineStr">
+      <c r="I8" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I8" s="22" t="n">
+      <c r="J8" s="22" t="n">
         <v>0.0207</v>
       </c>
-      <c r="J8" s="22" t="n">
+      <c r="K8" s="22" t="n">
         <v>0.02</v>
       </c>
-      <c r="K8" s="22" t="n">
+      <c r="L8" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L8" s="20" t="inlineStr">
+      <c r="M8" s="20" t="inlineStr">
         <is>
           <t>创业板人工智能ETF 159381</t>
         </is>
       </c>
-      <c r="M8" s="23" t="n">
+      <c r="N8" s="23" t="n">
         <v>265305</v>
       </c>
-      <c r="N8" s="22" t="n">
+      <c r="O8" s="22" t="n">
         <v>0.07552791135270751</v>
       </c>
-      <c r="O8" s="21" t="inlineStr">
+      <c r="P8" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P8" s="21" t="inlineStr">
+      <c r="Q8" s="21" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q8" s="24" t="n"/>
-      <c r="R8" s="21" t="n">
+      <c r="R8" s="24" t="n"/>
+      <c r="S8" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S8" s="21" t="inlineStr">
+      <c r="T8" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T8" s="20" t="inlineStr">
+      <c r="U8" s="20" t="inlineStr">
         <is>
           <t>超目标 0.07%</t>
         </is>
       </c>
-      <c r="U8" s="25" t="n">
+      <c r="V8" s="25" t="n">
         <v>1.445</v>
       </c>
-      <c r="V8" s="26" t="n"/>
-      <c r="W8" s="21" t="n"/>
-      <c r="X8" s="26" t="n"/>
-      <c r="Y8" s="21" t="inlineStr">
+      <c r="W8" s="26" t="n"/>
+      <c r="X8" s="21" t="n"/>
+      <c r="Y8" s="26" t="n"/>
+      <c r="Z8" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z8" s="20" t="inlineStr">
+      <c r="AA8" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA8" s="21" t="inlineStr">
+      <c r="AB8" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB8" s="21" t="inlineStr">
+      <c r="AC8" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC8" s="21" t="inlineStr">
+      <c r="AD8" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD8" s="20" t="inlineStr">
+      <c r="AE8" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE8" s="20" t="inlineStr">
+      <c r="AF8" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF8" s="20" t="inlineStr">
+      <c r="AG8" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG8" s="20" t="inlineStr">
+      <c r="AH8" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH8" s="14" t="inlineStr">
+      <c r="AI8" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI8" s="20" t="inlineStr">
+      <c r="AJ8" s="20" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="AJ8" s="22" t="n">
+      <c r="AK8" s="22" t="n">
         <v>0.06</v>
       </c>
-      <c r="AK8" s="23" t="n">
+      <c r="AL8" s="23" t="n">
         <v>286980</v>
       </c>
-      <c r="AL8" s="23" t="n">
+      <c r="AM8" s="23" t="n">
         <v>21675</v>
       </c>
-      <c r="AM8" s="20" t="inlineStr">
+      <c r="AN8" s="20" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -12120,142 +12023,147 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
           <t>超目标 3.06%，禁止加仓</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="F9" s="13" t="n">
+      <c r="G9" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="H9" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H9" s="13" t="inlineStr">
+      <c r="I9" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I9" s="16" t="n">
+      <c r="J9" s="16" t="n">
         <v>0.0606</v>
       </c>
-      <c r="J9" s="16" t="n">
+      <c r="K9" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="K9" s="16" t="n">
+      <c r="L9" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="9" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>云计算ETF</t>
         </is>
       </c>
-      <c r="M9" s="17" t="n">
+      <c r="N9" s="17" t="n">
         <v>80146</v>
       </c>
-      <c r="N9" s="16" t="n">
+      <c r="O9" s="16" t="n">
         <v>0.4414523660185379</v>
       </c>
-      <c r="O9" s="13" t="inlineStr">
+      <c r="P9" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P9" s="13" t="inlineStr">
+      <c r="Q9" s="13" t="inlineStr">
         <is>
           <t>战术仓</t>
         </is>
       </c>
-      <c r="Q9" s="27" t="n"/>
-      <c r="R9" s="13" t="n">
+      <c r="R9" s="27" t="n"/>
+      <c r="S9" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S9" s="13" t="inlineStr">
+      <c r="T9" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T9" s="9" t="inlineStr">
+      <c r="U9" s="9" t="inlineStr">
         <is>
           <t>超目标 3.06%</t>
         </is>
       </c>
-      <c r="U9" s="28" t="n">
+      <c r="V9" s="28" t="n">
         <v>1.712</v>
       </c>
-      <c r="V9" s="29" t="n"/>
-      <c r="W9" s="13" t="n"/>
-      <c r="X9" s="29" t="n"/>
-      <c r="Y9" s="13" t="inlineStr">
+      <c r="W9" s="29" t="n"/>
+      <c r="X9" s="13" t="n"/>
+      <c r="Y9" s="29" t="n"/>
+      <c r="Z9" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z9" s="9" t="inlineStr">
+      <c r="AA9" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA9" s="13" t="inlineStr">
+      <c r="AB9" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB9" s="13" t="inlineStr">
+      <c r="AC9" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC9" s="13" t="inlineStr">
+      <c r="AD9" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD9" s="9" t="inlineStr">
+      <c r="AE9" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE9" s="9" t="inlineStr">
+      <c r="AF9" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF9" s="9" t="inlineStr">
+      <c r="AG9" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG9" s="9" t="inlineStr">
+      <c r="AH9" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH9" s="14" t="inlineStr">
+      <c r="AI9" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI9" s="9" t="inlineStr">
+      <c r="AJ9" s="9" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="AJ9" s="16" t="n">
+      <c r="AK9" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="AK9" s="17" t="n">
+      <c r="AL9" s="17" t="n">
         <v>143490</v>
       </c>
-      <c r="AL9" s="17" t="n">
+      <c r="AM9" s="17" t="n">
         <v>63344</v>
       </c>
-      <c r="AM9" s="9" t="inlineStr">
+      <c r="AN9" s="9" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -12279,142 +12187,147 @@
       </c>
       <c r="D10" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
           <t>超目标 1.02%，禁止加仓</t>
         </is>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="F10" s="21" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="G10" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="H10" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H10" s="21" t="inlineStr">
+      <c r="I10" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I10" s="22" t="n">
+      <c r="J10" s="22" t="n">
         <v>0.0702</v>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="K10" s="22" t="n">
         <v>0.06</v>
       </c>
-      <c r="K10" s="22" t="n">
+      <c r="L10" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L10" s="20" t="inlineStr">
+      <c r="M10" s="20" t="inlineStr">
         <is>
           <t>中证A500ETF</t>
         </is>
       </c>
-      <c r="M10" s="23" t="n">
+      <c r="N10" s="23" t="n">
         <v>273365.8</v>
       </c>
-      <c r="N10" s="22" t="n">
+      <c r="O10" s="22" t="n">
         <v>0.285579657118963</v>
       </c>
-      <c r="O10" s="21" t="inlineStr">
+      <c r="P10" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P10" s="21" t="inlineStr">
+      <c r="Q10" s="21" t="inlineStr">
         <is>
           <t>低波权益层</t>
         </is>
       </c>
-      <c r="Q10" s="24" t="n"/>
-      <c r="R10" s="21" t="n">
+      <c r="R10" s="24" t="n"/>
+      <c r="S10" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S10" s="21" t="inlineStr">
+      <c r="T10" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T10" s="20" t="inlineStr">
+      <c r="U10" s="20" t="inlineStr">
         <is>
           <t>超目标 1.02%</t>
         </is>
       </c>
-      <c r="U10" s="25" t="n">
+      <c r="V10" s="25" t="n">
         <v>1.323</v>
       </c>
-      <c r="V10" s="26" t="n"/>
-      <c r="W10" s="21" t="n"/>
-      <c r="X10" s="26" t="n"/>
-      <c r="Y10" s="21" t="inlineStr">
+      <c r="W10" s="26" t="n"/>
+      <c r="X10" s="21" t="n"/>
+      <c r="Y10" s="26" t="n"/>
+      <c r="Z10" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z10" s="20" t="inlineStr">
+      <c r="AA10" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA10" s="21" t="inlineStr">
+      <c r="AB10" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB10" s="21" t="inlineStr">
+      <c r="AC10" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC10" s="21" t="inlineStr">
+      <c r="AD10" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD10" s="20" t="inlineStr">
+      <c r="AE10" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE10" s="20" t="inlineStr">
+      <c r="AF10" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF10" s="20" t="inlineStr">
+      <c r="AG10" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG10" s="20" t="inlineStr">
+      <c r="AH10" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH10" s="14" t="inlineStr">
+      <c r="AI10" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI10" s="20" t="inlineStr">
+      <c r="AJ10" s="20" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="AJ10" s="22" t="n">
+      <c r="AK10" s="22" t="n">
         <v>0.08</v>
       </c>
-      <c r="AK10" s="23" t="n">
+      <c r="AL10" s="23" t="n">
         <v>382640</v>
       </c>
-      <c r="AL10" s="23" t="n">
+      <c r="AM10" s="23" t="n">
         <v>109274.2</v>
       </c>
-      <c r="AM10" s="20" t="inlineStr">
+      <c r="AN10" s="20" t="inlineStr">
         <is>
           <t>配置中</t>
         </is>
@@ -12438,138 +12351,143 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E11" s="9" t="inlineStr">
+        <is>
           <t>超目标 1.41%，禁止加仓</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="F11" s="13" t="n">
+      <c r="G11" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="H11" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H11" s="13" t="inlineStr">
+      <c r="I11" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I11" s="16" t="n">
+      <c r="J11" s="16" t="n">
         <v>0.0541</v>
       </c>
-      <c r="J11" s="16" t="n">
+      <c r="K11" s="16" t="n">
         <v>0.04</v>
       </c>
-      <c r="K11" s="16" t="n">
+      <c r="L11" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L11" s="9" t="n"/>
-      <c r="M11" s="17" t="n">
-        <v/>
-      </c>
-      <c r="N11" s="16" t="n">
-        <v/>
-      </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="17" t="n">
+        <v/>
+      </c>
+      <c r="O11" s="16" t="n">
+        <v/>
+      </c>
+      <c r="P11" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P11" s="13" t="inlineStr">
+      <c r="Q11" s="13" t="inlineStr">
         <is>
           <t>纯防御层</t>
         </is>
       </c>
-      <c r="Q11" s="27" t="n"/>
-      <c r="R11" s="13" t="n">
+      <c r="R11" s="27" t="n"/>
+      <c r="S11" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S11" s="13" t="inlineStr">
+      <c r="T11" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T11" s="9" t="inlineStr">
+      <c r="U11" s="9" t="inlineStr">
         <is>
           <t>超目标 1.41%</t>
         </is>
       </c>
-      <c r="U11" s="28" t="n">
+      <c r="V11" s="28" t="n">
         <v>141.388</v>
       </c>
-      <c r="V11" s="29" t="n"/>
-      <c r="W11" s="13" t="n"/>
-      <c r="X11" s="29" t="n"/>
-      <c r="Y11" s="13" t="inlineStr">
+      <c r="W11" s="29" t="n"/>
+      <c r="X11" s="13" t="n"/>
+      <c r="Y11" s="29" t="n"/>
+      <c r="Z11" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z11" s="9" t="inlineStr">
+      <c r="AA11" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA11" s="13" t="inlineStr">
+      <c r="AB11" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB11" s="13" t="inlineStr">
+      <c r="AC11" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC11" s="13" t="inlineStr">
+      <c r="AD11" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD11" s="9" t="inlineStr">
+      <c r="AE11" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE11" s="9" t="inlineStr">
+      <c r="AF11" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF11" s="9" t="inlineStr">
+      <c r="AG11" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG11" s="9" t="inlineStr">
+      <c r="AH11" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH11" s="14" t="inlineStr">
+      <c r="AI11" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI11" s="9" t="inlineStr">
+      <c r="AJ11" s="9" t="inlineStr">
         <is>
           <t>当前仓位已达或超过目标仓位</t>
         </is>
       </c>
-      <c r="AJ11" s="16" t="n">
-        <v/>
-      </c>
-      <c r="AK11" s="17" t="n">
+      <c r="AK11" s="16" t="n">
         <v/>
       </c>
       <c r="AL11" s="17" t="n">
         <v/>
       </c>
-      <c r="AM11" s="9" t="n"/>
+      <c r="AM11" s="17" t="n">
+        <v/>
+      </c>
+      <c r="AN11" s="9" t="n"/>
     </row>
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="18" t="inlineStr">
@@ -12589,142 +12507,147 @@
       </c>
       <c r="D12" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
           <t>遗留仓禁止新买；超目标 4.33%</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="F12" s="21" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="G12" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="H12" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="I12" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I12" s="22" t="n">
+      <c r="J12" s="22" t="n">
         <v>0.09329999999999999</v>
       </c>
-      <c r="J12" s="22" t="n">
+      <c r="K12" s="22" t="n">
         <v>0.05</v>
       </c>
-      <c r="K12" s="22" t="n">
+      <c r="L12" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L12" s="20" t="inlineStr">
+      <c r="M12" s="20" t="inlineStr">
         <is>
           <t>比亚迪+绿电+储能</t>
         </is>
       </c>
-      <c r="M12" s="23" t="n">
+      <c r="N12" s="23" t="n">
         <v>-48452.39999999999</v>
       </c>
-      <c r="N12" s="22" t="n">
+      <c r="O12" s="22" t="n">
         <v>1.337670917833995</v>
       </c>
-      <c r="O12" s="21" t="inlineStr">
+      <c r="P12" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P12" s="21" t="inlineStr">
+      <c r="Q12" s="21" t="inlineStr">
         <is>
           <t>遗留仓</t>
         </is>
       </c>
-      <c r="Q12" s="24" t="n"/>
-      <c r="R12" s="21" t="n">
+      <c r="R12" s="24" t="n"/>
+      <c r="S12" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S12" s="21" t="inlineStr">
+      <c r="T12" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T12" s="20" t="inlineStr">
+      <c r="U12" s="20" t="inlineStr">
         <is>
           <t>超目标 4.33%</t>
         </is>
       </c>
-      <c r="U12" s="25" t="n">
+      <c r="V12" s="25" t="n">
         <v>88.64</v>
       </c>
-      <c r="V12" s="26" t="n"/>
-      <c r="W12" s="21" t="n"/>
-      <c r="X12" s="26" t="n"/>
-      <c r="Y12" s="21" t="inlineStr">
+      <c r="W12" s="26" t="n"/>
+      <c r="X12" s="21" t="n"/>
+      <c r="Y12" s="26" t="n"/>
+      <c r="Z12" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z12" s="20" t="inlineStr">
+      <c r="AA12" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA12" s="21" t="inlineStr">
+      <c r="AB12" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB12" s="21" t="inlineStr">
+      <c r="AC12" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC12" s="21" t="inlineStr">
+      <c r="AD12" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD12" s="20" t="inlineStr">
+      <c r="AE12" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE12" s="20" t="inlineStr">
+      <c r="AF12" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF12" s="20" t="inlineStr">
+      <c r="AG12" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG12" s="20" t="inlineStr">
+      <c r="AH12" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH12" s="14" t="inlineStr">
+      <c r="AI12" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI12" s="20" t="inlineStr">
+      <c r="AJ12" s="20" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="AJ12" s="22" t="n">
+      <c r="AK12" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="AK12" s="23" t="n">
+      <c r="AL12" s="23" t="n">
         <v>143490</v>
       </c>
-      <c r="AL12" s="23" t="n">
+      <c r="AM12" s="23" t="n">
         <v>191942.4</v>
       </c>
-      <c r="AM12" s="20" t="inlineStr">
+      <c r="AN12" s="20" t="inlineStr">
         <is>
           <t>达到或超过年度目标</t>
         </is>
@@ -12748,138 +12671,143 @@
       </c>
       <c r="D13" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
           <t>遗留仓禁止新买；超目标 3.29%</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="F13" s="13" t="n">
+      <c r="G13" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="H13" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H13" s="13" t="inlineStr">
+      <c r="I13" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I13" s="16" t="n">
+      <c r="J13" s="16" t="n">
         <v>0.0529</v>
       </c>
-      <c r="J13" s="16" t="n">
+      <c r="K13" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="K13" s="16" t="n">
+      <c r="L13" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="9" t="n"/>
-      <c r="M13" s="17" t="n">
-        <v/>
-      </c>
-      <c r="N13" s="16" t="n">
-        <v/>
-      </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="M13" s="9" t="n"/>
+      <c r="N13" s="17" t="n">
+        <v/>
+      </c>
+      <c r="O13" s="16" t="n">
+        <v/>
+      </c>
+      <c r="P13" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P13" s="13" t="inlineStr">
+      <c r="Q13" s="13" t="inlineStr">
         <is>
           <t>遗留仓</t>
         </is>
       </c>
-      <c r="Q13" s="27" t="n"/>
-      <c r="R13" s="13" t="n">
+      <c r="R13" s="27" t="n"/>
+      <c r="S13" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S13" s="13" t="inlineStr">
+      <c r="T13" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T13" s="9" t="inlineStr">
+      <c r="U13" s="9" t="inlineStr">
         <is>
           <t>超目标 3.29%</t>
         </is>
       </c>
-      <c r="U13" s="28" t="n">
+      <c r="V13" s="28" t="n">
         <v>65.26000000000001</v>
       </c>
-      <c r="V13" s="29" t="n"/>
-      <c r="W13" s="13" t="n"/>
-      <c r="X13" s="29" t="n"/>
-      <c r="Y13" s="13" t="inlineStr">
+      <c r="W13" s="29" t="n"/>
+      <c r="X13" s="13" t="n"/>
+      <c r="Y13" s="29" t="n"/>
+      <c r="Z13" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z13" s="9" t="inlineStr">
+      <c r="AA13" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA13" s="13" t="inlineStr">
+      <c r="AB13" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB13" s="13" t="inlineStr">
+      <c r="AC13" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC13" s="13" t="inlineStr">
+      <c r="AD13" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD13" s="9" t="inlineStr">
+      <c r="AE13" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE13" s="9" t="inlineStr">
+      <c r="AF13" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF13" s="9" t="inlineStr">
+      <c r="AG13" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG13" s="9" t="inlineStr">
+      <c r="AH13" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH13" s="14" t="inlineStr">
+      <c r="AI13" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI13" s="9" t="inlineStr">
+      <c r="AJ13" s="9" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="AJ13" s="16" t="n">
-        <v/>
-      </c>
-      <c r="AK13" s="17" t="n">
+      <c r="AK13" s="16" t="n">
         <v/>
       </c>
       <c r="AL13" s="17" t="n">
         <v/>
       </c>
-      <c r="AM13" s="9" t="n"/>
+      <c r="AM13" s="17" t="n">
+        <v/>
+      </c>
+      <c r="AN13" s="9" t="n"/>
     </row>
     <row r="14" ht="38" customHeight="1">
       <c r="A14" s="18" t="inlineStr">
@@ -12899,142 +12827,147 @@
       </c>
       <c r="D14" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
           <t>遗留仓禁止新买；超目标 1.56%</t>
         </is>
       </c>
-      <c r="E14" s="21" t="inlineStr">
+      <c r="F14" s="21" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="G14" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="H14" s="20" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H14" s="21" t="inlineStr">
+      <c r="I14" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I14" s="22" t="n">
+      <c r="J14" s="22" t="n">
         <v>0.0456</v>
       </c>
-      <c r="J14" s="22" t="n">
+      <c r="K14" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="K14" s="22" t="n">
+      <c r="L14" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L14" s="20" t="inlineStr">
+      <c r="M14" s="20" t="inlineStr">
         <is>
           <t>比亚迪+绿电+储能</t>
         </is>
       </c>
-      <c r="M14" s="23" t="n">
+      <c r="N14" s="23" t="n">
         <v>-48452.39999999999</v>
       </c>
-      <c r="N14" s="22" t="n">
+      <c r="O14" s="22" t="n">
         <v>1.337670917833995</v>
       </c>
-      <c r="O14" s="21" t="inlineStr">
+      <c r="P14" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P14" s="21" t="inlineStr">
+      <c r="Q14" s="21" t="inlineStr">
         <is>
           <t>遗留仓</t>
         </is>
       </c>
-      <c r="Q14" s="24" t="n"/>
-      <c r="R14" s="21" t="n">
+      <c r="R14" s="24" t="n"/>
+      <c r="S14" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S14" s="21" t="inlineStr">
+      <c r="T14" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T14" s="20" t="inlineStr">
+      <c r="U14" s="20" t="inlineStr">
         <is>
           <t>超目标 1.56%</t>
         </is>
       </c>
-      <c r="U14" s="25" t="n">
+      <c r="V14" s="25" t="n">
         <v>1.19</v>
       </c>
-      <c r="V14" s="26" t="n"/>
-      <c r="W14" s="21" t="n"/>
-      <c r="X14" s="26" t="n"/>
-      <c r="Y14" s="21" t="inlineStr">
+      <c r="W14" s="26" t="n"/>
+      <c r="X14" s="21" t="n"/>
+      <c r="Y14" s="26" t="n"/>
+      <c r="Z14" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z14" s="20" t="inlineStr">
+      <c r="AA14" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA14" s="21" t="inlineStr">
+      <c r="AB14" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB14" s="21" t="inlineStr">
+      <c r="AC14" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC14" s="21" t="inlineStr">
+      <c r="AD14" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD14" s="20" t="inlineStr">
+      <c r="AE14" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE14" s="20" t="inlineStr">
+      <c r="AF14" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF14" s="20" t="inlineStr">
+      <c r="AG14" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG14" s="20" t="inlineStr">
+      <c r="AH14" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH14" s="14" t="inlineStr">
+      <c r="AI14" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI14" s="20" t="inlineStr">
+      <c r="AJ14" s="20" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="AJ14" s="22" t="n">
+      <c r="AK14" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="AK14" s="23" t="n">
+      <c r="AL14" s="23" t="n">
         <v>143490</v>
       </c>
-      <c r="AL14" s="23" t="n">
+      <c r="AM14" s="23" t="n">
         <v>191942.4</v>
       </c>
-      <c r="AM14" s="20" t="inlineStr">
+      <c r="AN14" s="20" t="inlineStr">
         <is>
           <t>达到或超过年度目标</t>
         </is>
@@ -13058,142 +12991,147 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
           <t>遗留仓禁止新买；超目标 2.48%</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="F15" s="13" t="n">
+      <c r="G15" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="H15" s="9" t="inlineStr">
         <is>
           <t>数据不足，需人工评分</t>
         </is>
       </c>
-      <c r="H15" s="13" t="inlineStr">
+      <c r="I15" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I15" s="16" t="n">
+      <c r="J15" s="16" t="n">
         <v>0.0448</v>
       </c>
-      <c r="J15" s="16" t="n">
+      <c r="K15" s="16" t="n">
         <v>0.02</v>
       </c>
-      <c r="K15" s="16" t="n">
+      <c r="L15" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="L15" s="9" t="inlineStr">
+      <c r="M15" s="9" t="inlineStr">
         <is>
           <t>比亚迪+绿电+储能</t>
         </is>
       </c>
-      <c r="M15" s="17" t="n">
+      <c r="N15" s="17" t="n">
         <v>-48452.39999999999</v>
       </c>
-      <c r="N15" s="16" t="n">
+      <c r="O15" s="16" t="n">
         <v>1.337670917833995</v>
       </c>
-      <c r="O15" s="13" t="inlineStr">
+      <c r="P15" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P15" s="13" t="inlineStr">
+      <c r="Q15" s="13" t="inlineStr">
         <is>
           <t>遗留仓</t>
         </is>
       </c>
-      <c r="Q15" s="27" t="n"/>
-      <c r="R15" s="13" t="n">
+      <c r="R15" s="27" t="n"/>
+      <c r="S15" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S15" s="13" t="inlineStr">
+      <c r="T15" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T15" s="9" t="inlineStr">
+      <c r="U15" s="9" t="inlineStr">
         <is>
           <t>超目标 2.48%</t>
         </is>
       </c>
-      <c r="U15" s="28" t="n">
+      <c r="V15" s="28" t="n">
         <v>2.296</v>
       </c>
-      <c r="V15" s="29" t="n"/>
-      <c r="W15" s="13" t="n"/>
-      <c r="X15" s="29" t="n"/>
-      <c r="Y15" s="13" t="inlineStr">
+      <c r="W15" s="29" t="n"/>
+      <c r="X15" s="13" t="n"/>
+      <c r="Y15" s="29" t="n"/>
+      <c r="Z15" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z15" s="9" t="inlineStr">
+      <c r="AA15" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA15" s="13" t="inlineStr">
+      <c r="AB15" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB15" s="13" t="inlineStr">
+      <c r="AC15" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC15" s="13" t="inlineStr">
+      <c r="AD15" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD15" s="9" t="inlineStr">
+      <c r="AE15" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE15" s="9" t="inlineStr">
+      <c r="AF15" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF15" s="9" t="inlineStr">
+      <c r="AG15" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG15" s="9" t="inlineStr">
+      <c r="AH15" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH15" s="14" t="inlineStr">
+      <c r="AI15" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI15" s="9" t="inlineStr">
+      <c r="AJ15" s="9" t="inlineStr">
         <is>
           <t>遗留仓禁止新买，按减仓/退出纪律处理</t>
         </is>
       </c>
-      <c r="AJ15" s="16" t="n">
+      <c r="AK15" s="16" t="n">
         <v>0.03</v>
       </c>
-      <c r="AK15" s="17" t="n">
+      <c r="AL15" s="17" t="n">
         <v>143490</v>
       </c>
-      <c r="AL15" s="17" t="n">
+      <c r="AM15" s="17" t="n">
         <v>191942.4</v>
       </c>
-      <c r="AM15" s="9" t="inlineStr">
+      <c r="AN15" s="9" t="inlineStr">
         <is>
           <t>达到或超过年度目标</t>
         </is>
@@ -13217,138 +13155,143 @@
       </c>
       <c r="D16" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
           <t>指数锚点，仅观察，不执行买入</t>
         </is>
       </c>
-      <c r="E16" s="21" t="inlineStr">
+      <c r="F16" s="21" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="G16" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="H16" s="20" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="H16" s="21" t="inlineStr">
+      <c r="I16" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I16" s="22" t="n">
-        <v/>
-      </c>
       <c r="J16" s="22" t="n">
         <v/>
       </c>
       <c r="K16" s="22" t="n">
         <v/>
       </c>
-      <c r="L16" s="20" t="n"/>
-      <c r="M16" s="23" t="n">
-        <v/>
-      </c>
-      <c r="N16" s="22" t="n">
-        <v/>
-      </c>
-      <c r="O16" s="21" t="inlineStr">
+      <c r="L16" s="22" t="n">
+        <v/>
+      </c>
+      <c r="M16" s="20" t="n"/>
+      <c r="N16" s="23" t="n">
+        <v/>
+      </c>
+      <c r="O16" s="22" t="n">
+        <v/>
+      </c>
+      <c r="P16" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P16" s="21" t="inlineStr">
+      <c r="Q16" s="21" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q16" s="24" t="n"/>
-      <c r="R16" s="21" t="n">
+      <c r="R16" s="24" t="n"/>
+      <c r="S16" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S16" s="21" t="inlineStr">
+      <c r="T16" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T16" s="20" t="inlineStr">
+      <c r="U16" s="20" t="inlineStr">
         <is>
           <t>指数锚点（不可交易）</t>
         </is>
       </c>
-      <c r="U16" s="25" t="n">
-        <v/>
-      </c>
-      <c r="V16" s="26" t="n"/>
-      <c r="W16" s="21" t="n"/>
-      <c r="X16" s="26" t="n"/>
-      <c r="Y16" s="21" t="inlineStr">
+      <c r="V16" s="25" t="n">
+        <v/>
+      </c>
+      <c r="W16" s="26" t="n"/>
+      <c r="X16" s="21" t="n"/>
+      <c r="Y16" s="26" t="n"/>
+      <c r="Z16" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z16" s="20" t="inlineStr">
+      <c r="AA16" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA16" s="21" t="inlineStr">
+      <c r="AB16" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB16" s="21" t="inlineStr">
+      <c r="AC16" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC16" s="21" t="inlineStr">
+      <c r="AD16" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD16" s="20" t="inlineStr">
+      <c r="AE16" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE16" s="20" t="inlineStr">
+      <c r="AF16" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF16" s="20" t="inlineStr">
+      <c r="AG16" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG16" s="20" t="inlineStr">
+      <c r="AH16" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH16" s="14" t="inlineStr">
+      <c r="AI16" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI16" s="20" t="inlineStr">
+      <c r="AJ16" s="20" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="AJ16" s="22" t="n">
-        <v/>
-      </c>
-      <c r="AK16" s="23" t="n">
+      <c r="AK16" s="22" t="n">
         <v/>
       </c>
       <c r="AL16" s="23" t="n">
         <v/>
       </c>
-      <c r="AM16" s="20" t="n"/>
+      <c r="AM16" s="23" t="n">
+        <v/>
+      </c>
+      <c r="AN16" s="20" t="n"/>
     </row>
     <row r="17" ht="38" customHeight="1">
       <c r="A17" s="18" t="inlineStr">
@@ -13368,138 +13311,143 @@
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
           <t>指数锚点，仅观察，不执行买入</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="F17" s="13" t="n">
+      <c r="G17" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="H17" s="9" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="H17" s="13" t="inlineStr">
+      <c r="I17" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I17" s="16" t="n">
-        <v/>
-      </c>
       <c r="J17" s="16" t="n">
         <v/>
       </c>
       <c r="K17" s="16" t="n">
         <v/>
       </c>
-      <c r="L17" s="9" t="n"/>
-      <c r="M17" s="17" t="n">
-        <v/>
-      </c>
-      <c r="N17" s="16" t="n">
-        <v/>
-      </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="L17" s="16" t="n">
+        <v/>
+      </c>
+      <c r="M17" s="9" t="n"/>
+      <c r="N17" s="17" t="n">
+        <v/>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v/>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P17" s="13" t="inlineStr">
+      <c r="Q17" s="13" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q17" s="27" t="n"/>
-      <c r="R17" s="13" t="n">
+      <c r="R17" s="27" t="n"/>
+      <c r="S17" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S17" s="13" t="inlineStr">
+      <c r="T17" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T17" s="9" t="inlineStr">
+      <c r="U17" s="9" t="inlineStr">
         <is>
           <t>指数锚点（不可交易）</t>
         </is>
       </c>
-      <c r="U17" s="28" t="n">
-        <v/>
-      </c>
-      <c r="V17" s="29" t="n"/>
-      <c r="W17" s="13" t="n"/>
-      <c r="X17" s="29" t="n"/>
-      <c r="Y17" s="13" t="inlineStr">
+      <c r="V17" s="28" t="n">
+        <v/>
+      </c>
+      <c r="W17" s="29" t="n"/>
+      <c r="X17" s="13" t="n"/>
+      <c r="Y17" s="29" t="n"/>
+      <c r="Z17" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z17" s="9" t="inlineStr">
+      <c r="AA17" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA17" s="13" t="inlineStr">
+      <c r="AB17" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB17" s="13" t="inlineStr">
+      <c r="AC17" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC17" s="13" t="inlineStr">
+      <c r="AD17" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD17" s="9" t="inlineStr">
+      <c r="AE17" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE17" s="9" t="inlineStr">
+      <c r="AF17" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF17" s="9" t="inlineStr">
+      <c r="AG17" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG17" s="9" t="inlineStr">
+      <c r="AH17" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH17" s="14" t="inlineStr">
+      <c r="AI17" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI17" s="9" t="inlineStr">
+      <c r="AJ17" s="9" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="AJ17" s="16" t="n">
-        <v/>
-      </c>
-      <c r="AK17" s="17" t="n">
+      <c r="AK17" s="16" t="n">
         <v/>
       </c>
       <c r="AL17" s="17" t="n">
         <v/>
       </c>
-      <c r="AM17" s="9" t="n"/>
+      <c r="AM17" s="17" t="n">
+        <v/>
+      </c>
+      <c r="AN17" s="9" t="n"/>
     </row>
     <row r="18" ht="38" customHeight="1">
       <c r="A18" s="18" t="inlineStr">
@@ -13519,138 +13467,143 @@
       </c>
       <c r="D18" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
           <t>指数锚点，仅观察，不执行买入</t>
         </is>
       </c>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="F18" s="21" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="F18" s="21" t="n">
+      <c r="G18" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="20" t="inlineStr">
+      <c r="H18" s="20" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="H18" s="21" t="inlineStr">
+      <c r="I18" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I18" s="22" t="n">
-        <v/>
-      </c>
       <c r="J18" s="22" t="n">
         <v/>
       </c>
       <c r="K18" s="22" t="n">
         <v/>
       </c>
-      <c r="L18" s="20" t="n"/>
-      <c r="M18" s="23" t="n">
-        <v/>
-      </c>
-      <c r="N18" s="22" t="n">
-        <v/>
-      </c>
-      <c r="O18" s="21" t="inlineStr">
+      <c r="L18" s="22" t="n">
+        <v/>
+      </c>
+      <c r="M18" s="20" t="n"/>
+      <c r="N18" s="23" t="n">
+        <v/>
+      </c>
+      <c r="O18" s="22" t="n">
+        <v/>
+      </c>
+      <c r="P18" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P18" s="21" t="inlineStr">
+      <c r="Q18" s="21" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q18" s="24" t="n"/>
-      <c r="R18" s="21" t="n">
+      <c r="R18" s="24" t="n"/>
+      <c r="S18" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S18" s="21" t="inlineStr">
+      <c r="T18" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T18" s="20" t="inlineStr">
+      <c r="U18" s="20" t="inlineStr">
         <is>
           <t>指数锚点（不可交易）</t>
         </is>
       </c>
-      <c r="U18" s="25" t="n">
-        <v/>
-      </c>
-      <c r="V18" s="26" t="n"/>
-      <c r="W18" s="21" t="n"/>
-      <c r="X18" s="26" t="n"/>
-      <c r="Y18" s="21" t="inlineStr">
+      <c r="V18" s="25" t="n">
+        <v/>
+      </c>
+      <c r="W18" s="26" t="n"/>
+      <c r="X18" s="21" t="n"/>
+      <c r="Y18" s="26" t="n"/>
+      <c r="Z18" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z18" s="20" t="inlineStr">
+      <c r="AA18" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA18" s="21" t="inlineStr">
+      <c r="AB18" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB18" s="21" t="inlineStr">
+      <c r="AC18" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC18" s="21" t="inlineStr">
+      <c r="AD18" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD18" s="20" t="inlineStr">
+      <c r="AE18" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE18" s="20" t="inlineStr">
+      <c r="AF18" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF18" s="20" t="inlineStr">
+      <c r="AG18" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG18" s="20" t="inlineStr">
+      <c r="AH18" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH18" s="14" t="inlineStr">
+      <c r="AI18" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI18" s="20" t="inlineStr">
+      <c r="AJ18" s="20" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="AJ18" s="22" t="n">
-        <v/>
-      </c>
-      <c r="AK18" s="23" t="n">
+      <c r="AK18" s="22" t="n">
         <v/>
       </c>
       <c r="AL18" s="23" t="n">
         <v/>
       </c>
-      <c r="AM18" s="20" t="n"/>
+      <c r="AM18" s="23" t="n">
+        <v/>
+      </c>
+      <c r="AN18" s="20" t="n"/>
     </row>
     <row r="19" ht="38" customHeight="1">
       <c r="A19" s="18" t="inlineStr">
@@ -13670,138 +13623,143 @@
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
           <t>指数锚点，仅观察，不执行买入</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="F19" s="13" t="n">
+      <c r="G19" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="H19" s="9" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="H19" s="13" t="inlineStr">
+      <c r="I19" s="13" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I19" s="16" t="n">
-        <v/>
-      </c>
       <c r="J19" s="16" t="n">
         <v/>
       </c>
       <c r="K19" s="16" t="n">
         <v/>
       </c>
-      <c r="L19" s="9" t="n"/>
-      <c r="M19" s="17" t="n">
-        <v/>
-      </c>
-      <c r="N19" s="16" t="n">
-        <v/>
-      </c>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="L19" s="16" t="n">
+        <v/>
+      </c>
+      <c r="M19" s="9" t="n"/>
+      <c r="N19" s="17" t="n">
+        <v/>
+      </c>
+      <c r="O19" s="16" t="n">
+        <v/>
+      </c>
+      <c r="P19" s="13" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P19" s="13" t="inlineStr">
+      <c r="Q19" s="13" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q19" s="27" t="n"/>
-      <c r="R19" s="13" t="n">
+      <c r="R19" s="27" t="n"/>
+      <c r="S19" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="S19" s="13" t="inlineStr">
+      <c r="T19" s="13" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T19" s="9" t="inlineStr">
+      <c r="U19" s="9" t="inlineStr">
         <is>
           <t>指数锚点（不可交易）</t>
         </is>
       </c>
-      <c r="U19" s="28" t="n">
-        <v/>
-      </c>
-      <c r="V19" s="29" t="n"/>
-      <c r="W19" s="13" t="n"/>
-      <c r="X19" s="29" t="n"/>
-      <c r="Y19" s="13" t="inlineStr">
+      <c r="V19" s="28" t="n">
+        <v/>
+      </c>
+      <c r="W19" s="29" t="n"/>
+      <c r="X19" s="13" t="n"/>
+      <c r="Y19" s="29" t="n"/>
+      <c r="Z19" s="13" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z19" s="9" t="inlineStr">
+      <c r="AA19" s="9" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA19" s="13" t="inlineStr">
+      <c r="AB19" s="13" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB19" s="13" t="inlineStr">
+      <c r="AC19" s="13" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC19" s="13" t="inlineStr">
+      <c r="AD19" s="13" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD19" s="9" t="inlineStr">
+      <c r="AE19" s="9" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE19" s="9" t="inlineStr">
+      <c r="AF19" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF19" s="9" t="inlineStr">
+      <c r="AG19" s="9" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG19" s="9" t="inlineStr">
+      <c r="AH19" s="9" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH19" s="14" t="inlineStr">
+      <c r="AI19" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI19" s="9" t="inlineStr">
+      <c r="AJ19" s="9" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="AJ19" s="16" t="n">
-        <v/>
-      </c>
-      <c r="AK19" s="17" t="n">
+      <c r="AK19" s="16" t="n">
         <v/>
       </c>
       <c r="AL19" s="17" t="n">
         <v/>
       </c>
-      <c r="AM19" s="9" t="n"/>
+      <c r="AM19" s="17" t="n">
+        <v/>
+      </c>
+      <c r="AN19" s="9" t="n"/>
     </row>
     <row r="20" ht="38" customHeight="1">
       <c r="A20" s="18" t="inlineStr">
@@ -13821,141 +13779,146 @@
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
+          <t>暂不建议买入（行情未刷新或数据不完整）</t>
+        </is>
+      </c>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
           <t>指数锚点，仅观察，不执行买入</t>
         </is>
       </c>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="F20" s="21" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="F20" s="21" t="n">
+      <c r="G20" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="20" t="inlineStr">
+      <c r="H20" s="20" t="inlineStr">
         <is>
           <t>不适用</t>
         </is>
       </c>
-      <c r="H20" s="21" t="inlineStr">
+      <c r="I20" s="21" t="inlineStr">
         <is>
           <t>暂停标准新增</t>
         </is>
       </c>
-      <c r="I20" s="22" t="n">
-        <v/>
-      </c>
       <c r="J20" s="22" t="n">
         <v/>
       </c>
       <c r="K20" s="22" t="n">
         <v/>
       </c>
-      <c r="L20" s="20" t="n"/>
-      <c r="M20" s="23" t="n">
-        <v/>
-      </c>
-      <c r="N20" s="22" t="n">
-        <v/>
-      </c>
-      <c r="O20" s="21" t="inlineStr">
+      <c r="L20" s="22" t="n">
+        <v/>
+      </c>
+      <c r="M20" s="20" t="n"/>
+      <c r="N20" s="23" t="n">
+        <v/>
+      </c>
+      <c r="O20" s="22" t="n">
+        <v/>
+      </c>
+      <c r="P20" s="21" t="inlineStr">
         <is>
           <t>行情未刷新</t>
         </is>
       </c>
-      <c r="P20" s="21" t="inlineStr">
+      <c r="Q20" s="21" t="inlineStr">
         <is>
           <t>观察仓</t>
         </is>
       </c>
-      <c r="Q20" s="24" t="n"/>
-      <c r="R20" s="21" t="n">
+      <c r="R20" s="24" t="n"/>
+      <c r="S20" s="21" t="n">
         <v>1</v>
       </c>
-      <c r="S20" s="21" t="inlineStr">
+      <c r="T20" s="21" t="inlineStr">
         <is>
           <t>待确认</t>
         </is>
       </c>
-      <c r="T20" s="20" t="inlineStr">
+      <c r="U20" s="20" t="inlineStr">
         <is>
           <t>指数锚点（不可交易）</t>
         </is>
       </c>
-      <c r="U20" s="25" t="n">
-        <v/>
-      </c>
-      <c r="V20" s="26" t="n"/>
-      <c r="W20" s="21" t="n"/>
-      <c r="X20" s="26" t="n"/>
-      <c r="Y20" s="21" t="inlineStr">
+      <c r="V20" s="25" t="n">
+        <v/>
+      </c>
+      <c r="W20" s="26" t="n"/>
+      <c r="X20" s="21" t="n"/>
+      <c r="Y20" s="26" t="n"/>
+      <c r="Z20" s="21" t="inlineStr">
         <is>
           <t>缺少日内数据</t>
         </is>
       </c>
-      <c r="Z20" s="20" t="inlineStr">
+      <c r="AA20" s="20" t="inlineStr">
         <is>
           <t>缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AA20" s="21" t="inlineStr">
+      <c r="AB20" s="21" t="inlineStr">
         <is>
           <t>量能替代：缺少成交额/20日均额</t>
         </is>
       </c>
-      <c r="AB20" s="21" t="inlineStr">
+      <c r="AC20" s="21" t="inlineStr">
         <is>
           <t>折溢价替代：缺少涨跌幅</t>
         </is>
       </c>
-      <c r="AC20" s="21" t="inlineStr">
+      <c r="AD20" s="21" t="inlineStr">
         <is>
           <t>待人工确认</t>
         </is>
       </c>
-      <c r="AD20" s="20" t="inlineStr">
+      <c r="AE20" s="20" t="inlineStr">
         <is>
           <t>待次日确认</t>
         </is>
       </c>
-      <c r="AE20" s="20" t="inlineStr">
+      <c r="AF20" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AF20" s="20" t="inlineStr">
+      <c r="AG20" s="20" t="inlineStr">
         <is>
           <t>无</t>
         </is>
       </c>
-      <c r="AG20" s="20" t="inlineStr">
+      <c r="AH20" s="20" t="inlineStr">
         <is>
           <t>分时结构；量价关系；份额/筹码；折溢价/估值；龙头同步；次日验证</t>
         </is>
       </c>
-      <c r="AH20" s="14" t="inlineStr">
+      <c r="AI20" s="14" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="AI20" s="20" t="inlineStr">
+      <c r="AJ20" s="20" t="inlineStr">
         <is>
           <t>指数仅作市场锚点，不执行买入</t>
         </is>
       </c>
-      <c r="AJ20" s="22" t="n">
-        <v/>
-      </c>
-      <c r="AK20" s="23" t="n">
+      <c r="AK20" s="22" t="n">
         <v/>
       </c>
       <c r="AL20" s="23" t="n">
         <v/>
       </c>
-      <c r="AM20" s="20" t="n"/>
+      <c r="AM20" s="23" t="n">
+        <v/>
+      </c>
+      <c r="AN20" s="20" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AM20"/>
+  <autoFilter ref="A1:AN20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -16998,7 +16961,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>2026-06-20 16:08:19</t>
+          <t>2026-06-21 09:43:05</t>
         </is>
       </c>
     </row>

</xml_diff>